<commit_message>
reordered list of xlsx files
</commit_message>
<xml_diff>
--- a/results/Итог_все_результаты.xlsx
+++ b/results/Итог_все_результаты.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="поступенчатый_расчет_ступеней" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="расчет_ступеней_по_высоте_лопат" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Профилирование_лопаток" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Начальные_данные" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Начальные_данные" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="поступенчатый_расчет_ступеней" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="расчет_ступеней_по_высоте_лопат" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Профилирование_лопаток" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -554,6 +554,254 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Переменная</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Название (из комментария)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Параметры 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>d1_отн</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Диаметр относительный на входе</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.43</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>c_а1_отн</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Коэффициент расхода на входе</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>c_a2_отн</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Коэффициент расхода на выходе</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Hт_ср_отн</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Коэффициент напора в средних ступенях</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>H_т1</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Коэффициент напора в первой ступени</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>R_ср1</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Степень реактивности</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>D_type</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Форма проточной части</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>D_к_const</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Tа_полн</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Полная температура воздуха на входе</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Pа_полн</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Полное давление воздуха на входе</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>101300</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>G_в</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Расход воздуха</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>58.7</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>π_к_полн</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Полное повышение давления в компрессоре</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>18.2</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>n_ob_min</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>Число оборотов компрессора в мин</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>8600</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>R_в</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Газовая постоянная</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>287.4</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Показатель адиабаты воздуха</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3380,7 +3628,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5426,7 +5674,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8411,252 +8659,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="41" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Переменная</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Название (из комментария)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Параметры 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>d1_отн</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Диаметр относительный на входе</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>0.43</v>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>c_а1_отн</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Коэффициент расхода на входе</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>c_a2_отн</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Коэффициент расхода на выходе</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>0.36</v>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Hт_ср_отн</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>Коэффициент напора в средних ступенях</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>H_т1</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>Коэффициент напора в первой ступени</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>R_ср1</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>Степень реактивности</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>D_type</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>Форма проточной части</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>D_к_const</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Tа_полн</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>Полная температура воздуха на входе</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Pа_полн</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>Полное давление воздуха на входе</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>101300</v>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>G_в</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>Расход воздуха</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>58.7</v>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>π_к_полн</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>Полное повышение давления в компрессоре</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>18.2</v>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>n_ob_min</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>Число оборотов компрессора в мин</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>8600</v>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>R_в</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>Газовая постоянная</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>287.4</v>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>k</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>Показатель адиабаты воздуха</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>1.4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>